<commit_message>
fix: replace real reference numbers in parser testdata
Axis: credit card ref numbers (OKDKA8BO53PJGK etc.) were identical to
the real statement — replaced with TESTREF000000xX placeholders.
SBI: PMSBY reference numbers were near-identical to real ones (just
truncated); card fragment 652294 was real — replaced with clearly
fictional 999999*0000 and SBISB0999999... references. XLSX fixture
regenerated from the fixed CSV.
</commit_message>
<xml_diff>
--- a/internal/importer/parser/testdata/sbi_v1.xlsx
+++ b/internal/importer/parser/testdata/sbi_v1.xlsx
@@ -413,364 +413,153 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Mr. Rahul  Sharma</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>State Bank of India</t>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Ref No/Cheque No</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Balance</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SAMPLE STREET</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OPP.POST OFFICE</t>
-        </is>
+          <t xml:space="preserve"> DEP TFR SBI General Insurance Co Ltd SBIGEN 99900000001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="F2" t="n">
+        <v>14364.59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Date of Statement  :  10-05-2026</t>
+          <t>10/05/2025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Branch Code  :  9999</t>
-        </is>
+          <t xml:space="preserve"> WDL TFR PMSBY RENEWAL SBISB09999990000000001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F3" t="n">
+        <v>14344.59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Clear Balance  :  14454.59CR</t>
+          <t>25/06/2025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Branch Name  :  SAMPLE BRANCH</t>
-        </is>
+          <t xml:space="preserve"> INTEREST CREDIT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>97</v>
+      </c>
+      <c r="F4" t="n">
+        <v>14441.59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Uncleared Amount  :  0.00</t>
+          <t>19/09/2025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Branch Email ID  :  sbi.01222@sbi.co.in</t>
-        </is>
+          <t xml:space="preserve"> DEBIT ATMCard AMC 999999*0000</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>236</v>
+      </c>
+      <c r="F5" t="n">
+        <v>14205.59</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MOD Bal   :  0.00</t>
+          <t>25/09/2025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Branch Phone   :  0000000000</t>
-        </is>
+          <t xml:space="preserve"> INTEREST CREDIT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>91</v>
+      </c>
+      <c r="F6" t="n">
+        <v>14296.59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lien  :  0.00</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CIF Number  :  90000000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Limit  :  0.00</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Account Number  :  40000000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Monthly Avg Balance  :  0.00</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Product  :  Savings Account</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Interest Rate  :  2.50 % p.a.</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>IFSC Code  :  SBIN0001000</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Drawing Power  :  0.00</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Currency  :  INR</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Account Status  :  OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>CKYCR Number  :  30000000000000</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>MICR Code  :  000000000</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Account Open Date  :  26/08/2021</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Nominee  Name  :  XXXXXXXXXXX</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Statement From  :  01-04-2025  to  10-05-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Ref No/Cheque No</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>08/04/2025</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>DEP TFR SBI General Insurance Co Ltd</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>199.99</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>14364.59</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>10/05/2025</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>WDL TFR PMSBY RENEWAL SBISB01222</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>20.00</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>14344.59</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>25/06/2025</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>INTEREST CREDIT</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>97.00</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>14441.59</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>19/09/2025</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>DEBIT ATMCard AMC</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>236.00</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>14205.59</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>25/09/2025</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>INTEREST CREDIT</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>91.00</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>14296.59</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>09/05/2026</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>WDL TFR PMSBY RENEWAL SBISB01222</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>20.00</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>14454.59</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Statement Summary : 01-04-2025  To  10-05-2026</t>
-        </is>
+          <t xml:space="preserve"> WDL TFR PMSBY RENEWAL SBISB09999990000000002</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F7" t="n">
+        <v>14454.59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: replace specific amounts in parser testdata with round fictional values
Amounts like 9694.70, 236451.00, 199.99 were picked up from real
statements. Replaced with round numbers (5000, 200000, 200, etc.)
and recalculated balances to match.
</commit_message>
<xml_diff>
--- a/internal/importer/parser/testdata/sbi_v1.xlsx
+++ b/internal/importer/parser/testdata/sbi_v1.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,153 +413,204 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A2:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Ref No/Cheque No</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Balance</t>
-        </is>
-      </c>
-    </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Mr. Rahul  Sharma</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Account Number  :  999900000000001</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IFSC Code  :  SBIN0009999</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ref No/Cheque No</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>08/04/2025</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t xml:space="preserve"> DEP TFR SBI General Insurance Co Ltd SBIGEN 99900000001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="E2" t="n">
-        <v>199.99</v>
-      </c>
-      <c r="F2" t="n">
-        <v>14364.59</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 200.00</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>14200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>10/05/2025</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t xml:space="preserve"> WDL TFR PMSBY RENEWAL SBISB09999990000000001</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="F3" t="n">
-        <v>14344.59</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>14180.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>25/06/2025</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t xml:space="preserve"> INTEREST CREDIT</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="E4" t="n">
-        <v>97</v>
-      </c>
-      <c r="F4" t="n">
-        <v>14441.59</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>14280.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>19/09/2025</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t xml:space="preserve"> DEBIT ATMCard AMC 999999*0000</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="n">
-        <v>236</v>
-      </c>
-      <c r="F5" t="n">
-        <v>14205.59</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 200.00</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>14080.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>25/09/2025</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t xml:space="preserve"> INTEREST CREDIT</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="E6" t="n">
-        <v>91</v>
-      </c>
-      <c r="F6" t="n">
-        <v>14296.59</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>14180.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>09/05/2026</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t xml:space="preserve"> WDL TFR PMSBY RENEWAL SBISB09999990000000002</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="n">
-        <v>20</v>
-      </c>
-      <c r="F7" t="n">
-        <v>14454.59</v>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>14160.00</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>